<commit_message>
bottom panel drawing update
</commit_message>
<xml_diff>
--- a/BOM/Valkyrie V2 Build Guide.xlsx
+++ b/BOM/Valkyrie V2 Build Guide.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3837cd5b4a1a02ac/Document Library/GitHub/Project-Valkyrie/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10872" documentId="8_{5107759B-8870-48A8-933E-C4A7F6F41B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D9A92D6-2FA1-405A-9FEF-ECFBA5000332}"/>
+  <xr:revisionPtr revIDLastSave="10873" documentId="8_{5107759B-8870-48A8-933E-C4A7F6F41B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA6627CD-FF2C-4926-8AAE-C67853D688C7}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="11" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INDEX" sheetId="52" r:id="rId1"/>
@@ -8782,6 +8782,9 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="170" formatCode="[h]:mm:ss;@"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="169" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-en-150,1]hh:mm;@"/>
     </dxf>
     <dxf>
@@ -8791,13 +8794,14 @@
       <numFmt numFmtId="169" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-en-150,1]hh:mm;@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="[h]:mm:ss;@"/>
+      <numFmt numFmtId="165" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;_ ;_-@_ "/>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;_ ;_-@_ "/>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -8817,10 +8821,6 @@
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -8860,6 +8860,24 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -8968,29 +8986,8 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <font>
@@ -9009,6 +9006,9 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <font>
@@ -9067,9 +9067,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -9086,6 +9083,9 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <font>
@@ -9144,9 +9144,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -9163,6 +9160,9 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <font>
@@ -9221,9 +9221,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -9240,6 +9237,9 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <font>
@@ -9298,9 +9298,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -9317,6 +9314,9 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <font>
@@ -9375,15 +9375,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -9402,6 +9393,7 @@
       </font>
     </dxf>
     <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -9454,6 +9446,14 @@
       </font>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FF000000"/>
@@ -9504,15 +9504,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -9531,6 +9522,7 @@
       </font>
     </dxf>
     <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -9583,6 +9575,14 @@
       </font>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FF000000"/>
@@ -9617,15 +9617,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -9644,6 +9635,7 @@
       </font>
     </dxf>
     <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -9696,6 +9688,14 @@
       </font>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FF000000"/>
@@ -9730,9 +9730,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -9749,6 +9746,9 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <font>
@@ -10083,13 +10083,6 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="medium">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color indexed="64"/>
@@ -10114,6 +10107,13 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <fill>
@@ -10326,8 +10326,8 @@
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>323850</xdr:colOff>
       <xdr:row>195</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
@@ -11529,6 +11529,10 @@
 </namedSheetViews>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" connectionId="1" xr16:uid="{DBE9A247-92C8-4088-ACE5-271A69C73D57}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="3">
@@ -11541,7 +11545,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{1DE5977A-0070-4907-B3F1-83B3E9D3EAF9}" name="Table1321" displayName="Table1321" ref="A1:J157" totalsRowShown="0" headerRowDxfId="147" dataDxfId="146" headerRowBorderDxfId="144" tableBorderDxfId="145" headerRowCellStyle="Normal 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{1DE5977A-0070-4907-B3F1-83B3E9D3EAF9}" name="Table1321" displayName="Table1321" ref="A1:J157" totalsRowShown="0" headerRowDxfId="147" dataDxfId="145" headerRowBorderDxfId="146" tableBorderDxfId="144" headerRowCellStyle="Normal 2">
   <autoFilter ref="A1:J157" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J157">
     <sortCondition ref="A1:A157"/>
@@ -11573,7 +11577,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3C370705-9D71-4B07-907E-72DEACEAFBA2}" name="Part name" totalsRowDxfId="73" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
     <tableColumn id="7" xr3:uid="{D11DB86B-2519-40CE-A3B1-2DFF1E8D8BAF}" name="Description" totalsRowDxfId="72" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{030B0BC7-E7B6-43C0-9200-DE84B404D5FA}" name="BOM Quantity" dataDxfId="70" totalsRowDxfId="71" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
+    <tableColumn id="2" xr3:uid="{030B0BC7-E7B6-43C0-9200-DE84B404D5FA}" name="BOM Quantity" dataDxfId="71" totalsRowDxfId="70" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11588,7 +11592,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{FEDEBDB4-D2A0-4044-865C-6B89D3CC7592}" name="Part name" totalsRowDxfId="67" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
     <tableColumn id="7" xr3:uid="{4C265877-F081-4975-80F2-6B962EBD7F5B}" name="Description" totalsRowDxfId="66" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{C58356B1-645B-4209-9365-0DE732AD7AAF}" name="BOM Quantity" dataDxfId="64" totalsRowDxfId="65" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
+    <tableColumn id="2" xr3:uid="{C58356B1-645B-4209-9365-0DE732AD7AAF}" name="BOM Quantity" dataDxfId="65" totalsRowDxfId="64" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11601,20 +11605,20 @@
     <sortCondition ref="A1:A111"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C89F3025-C91C-4D89-A5CC-8772042DE324}" name="System" totalsRowLabel="Valkyrie V2" dataDxfId="61" totalsRowDxfId="62"/>
-    <tableColumn id="3" xr3:uid="{AE4E9077-B04D-4FB7-A226-807DE24B3CEE}" name="Filament Type" dataDxfId="59" totalsRowDxfId="60"/>
-    <tableColumn id="2" xr3:uid="{FCE9DC81-99C5-4DE1-AE60-3B3DE0EE8421}" name="Part" dataDxfId="57" totalsRowDxfId="58"/>
+    <tableColumn id="1" xr3:uid="{C89F3025-C91C-4D89-A5CC-8772042DE324}" name="System" totalsRowLabel="Valkyrie V2" dataDxfId="62" totalsRowDxfId="61"/>
+    <tableColumn id="3" xr3:uid="{AE4E9077-B04D-4FB7-A226-807DE24B3CEE}" name="Filament Type" dataDxfId="60" totalsRowDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{FCE9DC81-99C5-4DE1-AE60-3B3DE0EE8421}" name="Part" dataDxfId="58" totalsRowDxfId="57"/>
     <tableColumn id="6" xr3:uid="{672D19F0-1E84-4954-AA80-1A756FF64B85}" name="Weight" dataDxfId="56"/>
-    <tableColumn id="11" xr3:uid="{B345B84F-64A2-4E92-BB95-3C9B14E2A5EA}" name="QTY" totalsRowFunction="sum" dataDxfId="54" totalsRowDxfId="55" dataCellStyle="Normal 7"/>
-    <tableColumn id="4" xr3:uid="{8A449E36-4741-4576-8011-21C1B3D5DB29}" name="Weight Tot" totalsRowFunction="custom" dataDxfId="52" totalsRowDxfId="53" dataCellStyle="Normal 7">
+    <tableColumn id="11" xr3:uid="{B345B84F-64A2-4E92-BB95-3C9B14E2A5EA}" name="QTY" totalsRowFunction="sum" dataDxfId="55" totalsRowDxfId="54" dataCellStyle="Normal 7"/>
+    <tableColumn id="4" xr3:uid="{8A449E36-4741-4576-8011-21C1B3D5DB29}" name="Weight Tot" totalsRowFunction="custom" dataDxfId="53" totalsRowDxfId="52" dataCellStyle="Normal 7">
       <calculatedColumnFormula>SUM(Table6[[#This Row],[Weight]]*Table6[[#This Row],[QTY]])</calculatedColumnFormula>
       <totalsRowFormula>SUBTOTAL(109,Table6[Weight Tot])&amp;"g"</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{DF7CF065-4550-4DB7-B341-EF87320D0C8E}" name="Cost/part" totalsRowFunction="sum" dataDxfId="50" totalsRowDxfId="51">
+    <tableColumn id="9" xr3:uid="{DF7CF065-4550-4DB7-B341-EF87320D0C8E}" name="Cost/part" totalsRowFunction="sum" dataDxfId="51" totalsRowDxfId="50">
       <calculatedColumnFormula>$L$2/1000*Table6[[#This Row],[Weight]]*Table6[[#This Row],[QTY]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{84F519DD-FB90-4299-8700-857D723260B1}" name="Time/item" totalsRowFunction="sum" dataDxfId="48" totalsRowDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{CBC7571F-19BC-4246-AB6F-92AD07297E48}" name="Time Total" totalsRowFunction="sum" dataDxfId="46" totalsRowDxfId="47">
+    <tableColumn id="10" xr3:uid="{84F519DD-FB90-4299-8700-857D723260B1}" name="Time/item" totalsRowFunction="sum" dataDxfId="49" totalsRowDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{CBC7571F-19BC-4246-AB6F-92AD07297E48}" name="Time Total" totalsRowFunction="sum" dataDxfId="47" totalsRowDxfId="46">
       <calculatedColumnFormula>Table6[[#This Row],[Time/item]]*Table6[[#This Row],[QTY]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11798,7 +11802,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{C5533925-B810-4F05-9221-5D5DC08A3846}" name="Part name" totalsRowDxfId="124" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
     <tableColumn id="7" xr3:uid="{13C33B91-92BB-4F0B-8B89-D7D5416E5479}" name="Description" totalsRowDxfId="123" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{684CEE11-8A68-45FD-871F-FFCFA808FEBD}" name="BOM Quantity" dataDxfId="121" totalsRowDxfId="122" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
+    <tableColumn id="2" xr3:uid="{684CEE11-8A68-45FD-871F-FFCFA808FEBD}" name="BOM Quantity" dataDxfId="122" totalsRowDxfId="121" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11811,9 +11815,9 @@
     <sortCondition ref="B1:B59"/>
   </sortState>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{1CE47076-A60D-4220-8B3D-C6D4BAFB1164}" name="Part name" dataDxfId="116" totalsRowDxfId="117" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="7" xr3:uid="{D41EBA7C-1A32-4553-871C-D0C5C96C9E90}" name="Description" dataDxfId="114" totalsRowDxfId="115" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{1A8F0BE6-05F1-4339-9CFB-0F9B7B4E13D4}" name="BOM Quantity" dataDxfId="112" totalsRowDxfId="113" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
+    <tableColumn id="1" xr3:uid="{1CE47076-A60D-4220-8B3D-C6D4BAFB1164}" name="Part name" dataDxfId="117" totalsRowDxfId="116" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
+    <tableColumn id="7" xr3:uid="{D41EBA7C-1A32-4553-871C-D0C5C96C9E90}" name="Description" dataDxfId="115" totalsRowDxfId="114" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
+    <tableColumn id="2" xr3:uid="{1A8F0BE6-05F1-4339-9CFB-0F9B7B4E13D4}" name="BOM Quantity" dataDxfId="113" totalsRowDxfId="112" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11826,9 +11830,9 @@
     <sortCondition ref="B1:B33"/>
   </sortState>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{0F292740-142C-4538-B6E0-04426284E315}" name="Part name" dataDxfId="107" totalsRowDxfId="108" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="7" xr3:uid="{150C9F57-34E9-40EB-9D7E-4F2F4DC1A13F}" name="Description" dataDxfId="105" totalsRowDxfId="106" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{A7D6434D-4498-49EB-9D73-D244744029D3}" name="BOM Quantity" dataDxfId="103" totalsRowDxfId="104" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
+    <tableColumn id="1" xr3:uid="{0F292740-142C-4538-B6E0-04426284E315}" name="Part name" dataDxfId="108" totalsRowDxfId="107" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
+    <tableColumn id="7" xr3:uid="{150C9F57-34E9-40EB-9D7E-4F2F4DC1A13F}" name="Description" dataDxfId="106" totalsRowDxfId="105" totalsRowCellStyle="Normal 2"/>
+    <tableColumn id="2" xr3:uid="{A7D6434D-4498-49EB-9D73-D244744029D3}" name="BOM Quantity" dataDxfId="104" totalsRowDxfId="103" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11841,9 +11845,9 @@
     <sortCondition ref="B35:B44"/>
   </sortState>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B397B237-34CC-4F05-A03A-172D9B10CC01}" name="Part name" dataDxfId="98" totalsRowDxfId="99" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="7" xr3:uid="{A1AF3E5A-9878-43E6-8325-6EA13891B687}" name="Description" dataDxfId="96" totalsRowDxfId="97" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{1585E650-1008-4DC9-8D1C-8F6E78001D58}" name="BOM Quantity" dataDxfId="94" totalsRowDxfId="95" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
+    <tableColumn id="1" xr3:uid="{B397B237-34CC-4F05-A03A-172D9B10CC01}" name="Part name" dataDxfId="99" totalsRowDxfId="98" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
+    <tableColumn id="7" xr3:uid="{A1AF3E5A-9878-43E6-8325-6EA13891B687}" name="Description" dataDxfId="97" totalsRowDxfId="96" totalsRowCellStyle="Normal 2"/>
+    <tableColumn id="2" xr3:uid="{1585E650-1008-4DC9-8D1C-8F6E78001D58}" name="BOM Quantity" dataDxfId="95" totalsRowDxfId="94" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11858,7 +11862,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{E0A0C165-2589-4FA7-A356-93EEE88B2095}" name="Part name" totalsRowDxfId="91" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
     <tableColumn id="7" xr3:uid="{49376C16-406D-4D5F-8B92-3BFE5FB962B9}" name="Description" totalsRowDxfId="90" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{6252F354-5A67-4DD7-A1AA-3DADB5EF6BF7}" name="BOM Quantity" dataDxfId="88" totalsRowDxfId="89" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
+    <tableColumn id="2" xr3:uid="{6252F354-5A67-4DD7-A1AA-3DADB5EF6BF7}" name="BOM Quantity" dataDxfId="89" totalsRowDxfId="88" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11873,7 +11877,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D7153C23-8479-4254-BF69-2A4089CB71C0}" name="Part name" totalsRowDxfId="85" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
     <tableColumn id="7" xr3:uid="{5CF4E952-095C-46AE-A57F-99A26E57C478}" name="Description" totalsRowDxfId="84" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{8AE4D1C0-7F70-4D1E-B6EC-42038CE642DF}" name="BOM Quantity" dataDxfId="82" totalsRowDxfId="83" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
+    <tableColumn id="2" xr3:uid="{8AE4D1C0-7F70-4D1E-B6EC-42038CE642DF}" name="BOM Quantity" dataDxfId="83" totalsRowDxfId="82" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11888,7 +11892,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{DE5B6A3D-F02B-442F-8F0E-2D97466E9D55}" name="Part name" totalsRowDxfId="79" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
     <tableColumn id="7" xr3:uid="{CD84E571-7957-4B8F-9F34-DA3FA6BF0E23}" name="Description" totalsRowDxfId="78" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{52F63DEF-0CA0-45D5-85B8-E41A21AD2000}" name="BOM Quantity" dataDxfId="76" totalsRowDxfId="77" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
+    <tableColumn id="2" xr3:uid="{52F63DEF-0CA0-45D5-85B8-E41A21AD2000}" name="BOM Quantity" dataDxfId="77" totalsRowDxfId="76" dataCellStyle="Normal 2" totalsRowCellStyle="Normal 8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -19406,7 +19410,7 @@
     <col min="1" max="1" width="14.140625" style="83" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" style="83" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.42578125" style="83" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22" style="83" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" style="83" customWidth="1"/>
     <col min="5" max="5" width="15.85546875" style="83" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.7109375" style="83" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.42578125" style="93" bestFit="1" customWidth="1"/>
@@ -36136,5 +36140,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{104F2E57-B689-41C7-9E9B-C2B84A40008B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{104F2E57-B689-41C7-9E9B-C2B84A40008B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/DataMashup"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>